<commit_message>
implementation von frühester Zeitpunkt
</commit_message>
<xml_diff>
--- a/Data/Excel/Exports/Schueler_Zuweisungen.xlsx
+++ b/Data/Excel/Exports/Schueler_Zuweisungen.xlsx
@@ -1416,7 +1416,7 @@
         <v>147</v>
       </c>
       <c r="D11">
-        <v>8</v>
+        <v>20</v>
       </c>
       <c r="E11">
         <v>1</v>
@@ -1516,7 +1516,7 @@
         <v>148</v>
       </c>
       <c r="D16">
-        <v>17</v>
+        <v>6</v>
       </c>
       <c r="E16">
         <v>5</v>
@@ -1716,7 +1716,7 @@
         <v>150</v>
       </c>
       <c r="D26">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="E26">
         <v>5</v>
@@ -1916,7 +1916,7 @@
         <v>152</v>
       </c>
       <c r="D36">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="E36">
         <v>3</v>
@@ -2016,7 +2016,7 @@
         <v>153</v>
       </c>
       <c r="D41">
-        <v>27</v>
+        <v>17</v>
       </c>
       <c r="E41">
         <v>5</v>
@@ -2216,7 +2216,7 @@
         <v>155</v>
       </c>
       <c r="D51">
-        <v>21</v>
+        <v>2</v>
       </c>
       <c r="E51">
         <v>2</v>
@@ -2316,7 +2316,7 @@
         <v>156</v>
       </c>
       <c r="D56">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="E56">
         <v>5</v>
@@ -2796,10 +2796,10 @@
         <v>161</v>
       </c>
       <c r="D80">
-        <v>6</v>
+        <v>1</v>
       </c>
       <c r="E80">
-        <v>5</v>
+        <v>3</v>
       </c>
       <c r="F80" t="s">
         <v>276</v>
@@ -2816,10 +2816,10 @@
         <v>161</v>
       </c>
       <c r="D81">
-        <v>26</v>
+        <v>6</v>
       </c>
       <c r="E81">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F81" t="s">
         <v>276</v>
@@ -2916,7 +2916,7 @@
         <v>162</v>
       </c>
       <c r="D86">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="E86">
         <v>5</v>
@@ -3116,7 +3116,7 @@
         <v>164</v>
       </c>
       <c r="D96">
-        <v>10</v>
+        <v>15</v>
       </c>
       <c r="E96">
         <v>2</v>
@@ -3216,7 +3216,7 @@
         <v>165</v>
       </c>
       <c r="D101">
-        <v>14</v>
+        <v>22</v>
       </c>
       <c r="E101">
         <v>3</v>
@@ -3516,7 +3516,7 @@
         <v>168</v>
       </c>
       <c r="D116">
-        <v>27</v>
+        <v>6</v>
       </c>
       <c r="E116">
         <v>5</v>
@@ -3716,7 +3716,7 @@
         <v>169</v>
       </c>
       <c r="D126">
-        <v>16</v>
+        <v>27</v>
       </c>
       <c r="E126">
         <v>5</v>
@@ -3816,7 +3816,7 @@
         <v>170</v>
       </c>
       <c r="D131">
-        <v>3</v>
+        <v>16</v>
       </c>
       <c r="E131">
         <v>4</v>
@@ -4016,7 +4016,7 @@
         <v>172</v>
       </c>
       <c r="D141">
-        <v>26</v>
+        <v>19</v>
       </c>
       <c r="E141">
         <v>3</v>
@@ -4116,7 +4116,7 @@
         <v>173</v>
       </c>
       <c r="D146">
-        <v>2</v>
+        <v>26</v>
       </c>
       <c r="E146">
         <v>2</v>
@@ -4196,10 +4196,10 @@
         <v>174</v>
       </c>
       <c r="D150">
-        <v>25</v>
+        <v>23</v>
       </c>
       <c r="E150">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F150" t="s">
         <v>276</v>
@@ -4216,10 +4216,10 @@
         <v>174</v>
       </c>
       <c r="D151">
-        <v>20</v>
+        <v>15</v>
       </c>
       <c r="E151">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F151" t="s">
         <v>276</v>
@@ -4616,7 +4616,7 @@
         <v>178</v>
       </c>
       <c r="D171">
-        <v>4</v>
+        <v>23</v>
       </c>
       <c r="E171">
         <v>1</v>
@@ -4716,7 +4716,7 @@
         <v>179</v>
       </c>
       <c r="D176">
-        <v>14</v>
+        <v>4</v>
       </c>
       <c r="E176">
         <v>2</v>
@@ -4816,7 +4816,7 @@
         <v>180</v>
       </c>
       <c r="D181">
-        <v>13</v>
+        <v>3</v>
       </c>
       <c r="E181">
         <v>5</v>
@@ -5196,10 +5196,10 @@
         <v>184</v>
       </c>
       <c r="D200">
-        <v>27</v>
+        <v>14</v>
       </c>
       <c r="E200">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="F200" t="s">
         <v>276</v>
@@ -5216,10 +5216,10 @@
         <v>184</v>
       </c>
       <c r="D201">
-        <v>21</v>
+        <v>27</v>
       </c>
       <c r="E201">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="F201" t="s">
         <v>276</v>
@@ -5316,7 +5316,7 @@
         <v>185</v>
       </c>
       <c r="D206">
-        <v>6</v>
+        <v>16</v>
       </c>
       <c r="E206">
         <v>5</v>
@@ -5376,10 +5376,10 @@
         <v>186</v>
       </c>
       <c r="D209">
-        <v>6</v>
+        <v>25</v>
       </c>
       <c r="E209">
-        <v>5</v>
+        <v>2</v>
       </c>
       <c r="F209" t="s">
         <v>276</v>
@@ -5396,10 +5396,10 @@
         <v>186</v>
       </c>
       <c r="D210">
+        <v>7</v>
+      </c>
+      <c r="E210">
         <v>5</v>
-      </c>
-      <c r="E210">
-        <v>1</v>
       </c>
       <c r="F210" t="s">
         <v>276</v>
@@ -5416,10 +5416,10 @@
         <v>186</v>
       </c>
       <c r="D211">
-        <v>10</v>
+        <v>5</v>
       </c>
       <c r="E211">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="F211" t="s">
         <v>276</v>
@@ -5796,7 +5796,7 @@
         <v>190</v>
       </c>
       <c r="D230">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="E230">
         <v>5</v>
@@ -5816,7 +5816,7 @@
         <v>190</v>
       </c>
       <c r="D231">
-        <v>17</v>
+        <v>3</v>
       </c>
       <c r="E231">
         <v>4</v>
@@ -6016,7 +6016,7 @@
         <v>192</v>
       </c>
       <c r="D241">
-        <v>17</v>
+        <v>3</v>
       </c>
       <c r="E241">
         <v>5</v>
@@ -6316,7 +6316,7 @@
         <v>195</v>
       </c>
       <c r="D256">
-        <v>25</v>
+        <v>14</v>
       </c>
       <c r="E256">
         <v>2</v>
@@ -6496,10 +6496,10 @@
         <v>197</v>
       </c>
       <c r="D265">
-        <v>16</v>
+        <v>21</v>
       </c>
       <c r="E265">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F265" t="s">
         <v>276</v>
@@ -6516,10 +6516,10 @@
         <v>197</v>
       </c>
       <c r="D266">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="E266">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F266" t="s">
         <v>276</v>
@@ -6616,7 +6616,7 @@
         <v>198</v>
       </c>
       <c r="D271">
-        <v>3</v>
+        <v>17</v>
       </c>
       <c r="E271">
         <v>5</v>
@@ -6716,7 +6716,7 @@
         <v>199</v>
       </c>
       <c r="D276">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="E276">
         <v>3</v>
@@ -6896,7 +6896,7 @@
         <v>201</v>
       </c>
       <c r="D285">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="E285">
         <v>3</v>
@@ -7016,7 +7016,7 @@
         <v>202</v>
       </c>
       <c r="D291">
-        <v>3</v>
+        <v>17</v>
       </c>
       <c r="E291">
         <v>4</v>
@@ -7116,7 +7116,7 @@
         <v>203</v>
       </c>
       <c r="D296">
-        <v>7</v>
+        <v>3</v>
       </c>
       <c r="E296">
         <v>5</v>
@@ -7316,7 +7316,7 @@
         <v>205</v>
       </c>
       <c r="D306">
-        <v>2</v>
+        <v>5</v>
       </c>
       <c r="E306">
         <v>1</v>
@@ -7816,7 +7816,7 @@
         <v>210</v>
       </c>
       <c r="D331">
-        <v>12</v>
+        <v>16</v>
       </c>
       <c r="E331">
         <v>5</v>
@@ -8016,7 +8016,7 @@
         <v>212</v>
       </c>
       <c r="D341">
-        <v>4</v>
+        <v>20</v>
       </c>
       <c r="E341">
         <v>1</v>
@@ -8316,7 +8316,7 @@
         <v>215</v>
       </c>
       <c r="D356">
-        <v>14</v>
+        <v>4</v>
       </c>
       <c r="E356">
         <v>2</v>
@@ -8696,10 +8696,10 @@
         <v>218</v>
       </c>
       <c r="D375">
-        <v>10</v>
+        <v>6</v>
       </c>
       <c r="E375">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F375" t="s">
         <v>276</v>
@@ -8716,10 +8716,10 @@
         <v>218</v>
       </c>
       <c r="D376">
-        <v>11</v>
+        <v>4</v>
       </c>
       <c r="E376">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F376" t="s">
         <v>276</v>
@@ -9116,7 +9116,7 @@
         <v>221</v>
       </c>
       <c r="D396">
-        <v>25</v>
+        <v>4</v>
       </c>
       <c r="E396">
         <v>2</v>
@@ -9216,7 +9216,7 @@
         <v>222</v>
       </c>
       <c r="D401">
-        <v>22</v>
+        <v>14</v>
       </c>
       <c r="E401">
         <v>3</v>
@@ -9316,7 +9316,7 @@
         <v>223</v>
       </c>
       <c r="D406">
-        <v>25</v>
+        <v>21</v>
       </c>
       <c r="E406">
         <v>2</v>
@@ -9616,7 +9616,7 @@
         <v>226</v>
       </c>
       <c r="D421">
-        <v>19</v>
+        <v>22</v>
       </c>
       <c r="E421">
         <v>3</v>
@@ -9716,7 +9716,7 @@
         <v>181</v>
       </c>
       <c r="D426">
-        <v>10</v>
+        <v>26</v>
       </c>
       <c r="E426">
         <v>2</v>
@@ -9916,7 +9916,7 @@
         <v>228</v>
       </c>
       <c r="D436">
-        <v>17</v>
+        <v>16</v>
       </c>
       <c r="E436">
         <v>5</v>
@@ -10216,7 +10216,7 @@
         <v>231</v>
       </c>
       <c r="D451">
-        <v>12</v>
+        <v>3</v>
       </c>
       <c r="E451">
         <v>5</v>
@@ -10516,7 +10516,7 @@
         <v>234</v>
       </c>
       <c r="D466">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="E466">
         <v>3</v>
@@ -10616,7 +10616,7 @@
         <v>235</v>
       </c>
       <c r="D471">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="E471">
         <v>2</v>
@@ -10716,7 +10716,7 @@
         <v>236</v>
       </c>
       <c r="D476">
-        <v>21</v>
+        <v>2</v>
       </c>
       <c r="E476">
         <v>2</v>
@@ -10916,7 +10916,7 @@
         <v>238</v>
       </c>
       <c r="D486">
-        <v>2</v>
+        <v>25</v>
       </c>
       <c r="E486">
         <v>2</v>
@@ -11016,7 +11016,7 @@
         <v>239</v>
       </c>
       <c r="D491">
-        <v>26</v>
+        <v>25</v>
       </c>
       <c r="E491">
         <v>2</v>
@@ -11116,7 +11116,7 @@
         <v>240</v>
       </c>
       <c r="D496">
-        <v>7</v>
+        <v>17</v>
       </c>
       <c r="E496">
         <v>5</v>
@@ -11296,10 +11296,10 @@
         <v>242</v>
       </c>
       <c r="D505">
-        <v>6</v>
+        <v>21</v>
       </c>
       <c r="E505">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F505" t="s">
         <v>276</v>
@@ -11316,10 +11316,10 @@
         <v>242</v>
       </c>
       <c r="D506">
-        <v>25</v>
+        <v>22</v>
       </c>
       <c r="E506">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F506" t="s">
         <v>276</v>
@@ -11396,7 +11396,7 @@
         <v>243</v>
       </c>
       <c r="D510">
-        <v>22</v>
+        <v>9</v>
       </c>
       <c r="E510">
         <v>3</v>
@@ -11416,7 +11416,7 @@
         <v>243</v>
       </c>
       <c r="D511">
-        <v>11</v>
+        <v>6</v>
       </c>
       <c r="E511">
         <v>4</v>
@@ -11516,7 +11516,7 @@
         <v>244</v>
       </c>
       <c r="D516">
-        <v>16</v>
+        <v>3</v>
       </c>
       <c r="E516">
         <v>5</v>
@@ -11596,7 +11596,7 @@
         <v>245</v>
       </c>
       <c r="D520">
-        <v>22</v>
+        <v>6</v>
       </c>
       <c r="E520">
         <v>4</v>
@@ -11616,7 +11616,7 @@
         <v>245</v>
       </c>
       <c r="D521">
-        <v>1</v>
+        <v>14</v>
       </c>
       <c r="E521">
         <v>3</v>
@@ -12016,7 +12016,7 @@
         <v>249</v>
       </c>
       <c r="D541">
-        <v>17</v>
+        <v>12</v>
       </c>
       <c r="E541">
         <v>5</v>
@@ -12116,7 +12116,7 @@
         <v>250</v>
       </c>
       <c r="D546">
-        <v>2</v>
+        <v>15</v>
       </c>
       <c r="E546">
         <v>2</v>
@@ -12416,7 +12416,7 @@
         <v>253</v>
       </c>
       <c r="D561">
-        <v>16</v>
+        <v>3</v>
       </c>
       <c r="E561">
         <v>5</v>
@@ -12716,7 +12716,7 @@
         <v>256</v>
       </c>
       <c r="D576">
-        <v>3</v>
+        <v>16</v>
       </c>
       <c r="E576">
         <v>5</v>
@@ -12816,7 +12816,7 @@
         <v>257</v>
       </c>
       <c r="D581">
-        <v>17</v>
+        <v>11</v>
       </c>
       <c r="E581">
         <v>4</v>
@@ -13016,7 +13016,7 @@
         <v>259</v>
       </c>
       <c r="D591">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="E591">
         <v>3</v>
@@ -13516,7 +13516,7 @@
         <v>263</v>
       </c>
       <c r="D616">
-        <v>6</v>
+        <v>17</v>
       </c>
       <c r="E616">
         <v>5</v>
@@ -13616,7 +13616,7 @@
         <v>264</v>
       </c>
       <c r="D621">
-        <v>13</v>
+        <v>27</v>
       </c>
       <c r="E621">
         <v>5</v>
@@ -13716,7 +13716,7 @@
         <v>265</v>
       </c>
       <c r="D626">
-        <v>9</v>
+        <v>14</v>
       </c>
       <c r="E626">
         <v>3</v>
@@ -13816,7 +13816,7 @@
         <v>266</v>
       </c>
       <c r="D631">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="E631">
         <v>5</v>
@@ -13916,7 +13916,7 @@
         <v>267</v>
       </c>
       <c r="D636">
-        <v>17</v>
+        <v>27</v>
       </c>
       <c r="E636">
         <v>5</v>
@@ -14016,7 +14016,7 @@
         <v>268</v>
       </c>
       <c r="D641">
-        <v>25</v>
+        <v>4</v>
       </c>
       <c r="E641">
         <v>2</v>
@@ -14116,7 +14116,7 @@
         <v>20</v>
       </c>
       <c r="D646">
-        <v>12</v>
+        <v>17</v>
       </c>
       <c r="E646">
         <v>5</v>
@@ -14199,7 +14199,7 @@
         <v>17</v>
       </c>
       <c r="E650">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F650" t="s">
         <v>276</v>
@@ -14216,10 +14216,10 @@
         <v>269</v>
       </c>
       <c r="D651">
-        <v>6</v>
+        <v>12</v>
       </c>
       <c r="E651">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F651" t="s">
         <v>276</v>
@@ -14316,7 +14316,7 @@
         <v>270</v>
       </c>
       <c r="D656">
-        <v>22</v>
+        <v>6</v>
       </c>
       <c r="E656">
         <v>4</v>
@@ -14416,7 +14416,7 @@
         <v>271</v>
       </c>
       <c r="D661">
-        <v>1</v>
+        <v>19</v>
       </c>
       <c r="E661">
         <v>3</v>
@@ -14516,7 +14516,7 @@
         <v>272</v>
       </c>
       <c r="D666">
-        <v>8</v>
+        <v>14</v>
       </c>
       <c r="E666">
         <v>1</v>
@@ -14536,10 +14536,10 @@
         <v>273</v>
       </c>
       <c r="D667">
-        <v>25</v>
+        <v>14</v>
       </c>
       <c r="E667">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="F667" t="s">
         <v>276</v>
@@ -14556,10 +14556,10 @@
         <v>273</v>
       </c>
       <c r="D668">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="E668">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="F668" t="s">
         <v>276</v>
@@ -14576,10 +14576,10 @@
         <v>273</v>
       </c>
       <c r="D669">
-        <v>19</v>
+        <v>26</v>
       </c>
       <c r="E669">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F669" t="s">
         <v>276</v>
@@ -14596,10 +14596,10 @@
         <v>273</v>
       </c>
       <c r="D670">
-        <v>12</v>
+        <v>6</v>
       </c>
       <c r="E670">
-        <v>5</v>
+        <v>4</v>
       </c>
       <c r="F670" t="s">
         <v>276</v>
@@ -14616,10 +14616,10 @@
         <v>273</v>
       </c>
       <c r="D671">
-        <v>11</v>
+        <v>10</v>
       </c>
       <c r="E671">
-        <v>4</v>
+        <v>2</v>
       </c>
       <c r="F671" t="s">
         <v>276</v>
@@ -14656,10 +14656,10 @@
         <v>274</v>
       </c>
       <c r="D673">
-        <v>5</v>
+        <v>10</v>
       </c>
       <c r="E673">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F673" t="s">
         <v>276</v>
@@ -14676,10 +14676,10 @@
         <v>274</v>
       </c>
       <c r="D674">
-        <v>15</v>
+        <v>5</v>
       </c>
       <c r="E674">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F674" t="s">
         <v>276</v>
@@ -14696,7 +14696,7 @@
         <v>274</v>
       </c>
       <c r="D675">
-        <v>26</v>
+        <v>2</v>
       </c>
       <c r="E675">
         <v>2</v>
@@ -14716,7 +14716,7 @@
         <v>274</v>
       </c>
       <c r="D676">
-        <v>1</v>
+        <v>17</v>
       </c>
       <c r="E676">
         <v>4</v>

</xml_diff>